<commit_message>
fix(excel): separate swap collateral contexts
Bootstrap ESTR under EUR collateral instead of requiring an absent
EUR-under-USD collateral curve. Validate the generated worksheet
market inputs through the native Rust bootstrapper.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/swap_pricing_example.xlsx
+++ b/bindings/excel/examples/swap_pricing_example.xlsx
@@ -28,14 +28,15 @@
     <definedName name="Swap_Compounding">'1 Inputs'!$B$17</definedName>
     <definedName name="Swap_Context">'3 Build'!$B$7</definedName>
     <definedName name="Swap_Currency">'1 Inputs'!$B$13</definedName>
-    <definedName name="Swap_Curves">'2 Market'!$B$106</definedName>
     <definedName name="Swap_DayCounter">'1 Inputs'!$B$16</definedName>
-    <definedName name="Swap_EstrCurve">'3 Build'!$B$40</definedName>
+    <definedName name="Swap_EstrConfig">'2 Market'!$B$109</definedName>
+    <definedName name="Swap_EstrContext">'3 Build'!$B$10</definedName>
+    <definedName name="Swap_EstrCurve">'3 Build'!$B$43</definedName>
     <definedName name="Swap_EstrDiscount">'4 Results'!$B$14</definedName>
     <definedName name="Swap_EstrForward">'4 Results'!$B$16</definedName>
     <definedName name="Swap_EstrQuotes">'2 Market'!$A$18:$A$30</definedName>
-    <definedName name="Swap_Fair0">'3 Build'!$B$28</definedName>
-    <definedName name="Swap_Fair1">'3 Build'!$B$34</definedName>
+    <definedName name="Swap_Fair0">'3 Build'!$B$31</definedName>
+    <definedName name="Swap_Fair1">'3 Build'!$B$37</definedName>
     <definedName name="Swap_FairFixed">'4 Results'!$B$8</definedName>
     <definedName name="Swap_FairFloat">'4 Results'!$B$9</definedName>
     <definedName name="Swap_FixedFrequency">'1 Inputs'!$B$19</definedName>
@@ -43,12 +44,13 @@
     <definedName name="Swap_FloatFrequency">'1 Inputs'!$B$20</definedName>
     <definedName name="Swap_Index">'1 Inputs'!$B$14</definedName>
     <definedName name="Swap_InitialCurves">'2 Market'!$B$100</definedName>
+    <definedName name="Swap_InitialEstrCurves">'2 Market'!$B$106</definedName>
     <definedName name="Swap_InitialQuotes">'2 Market'!$B$34</definedName>
-    <definedName name="Swap_Instrument">'3 Build'!$B$10</definedName>
+    <definedName name="Swap_Instrument">'3 Build'!$B$13</definedName>
     <definedName name="Swap_Maturity">'1 Inputs'!$B$12</definedName>
     <definedName name="Swap_Notional">'1 Inputs'!$B$8</definedName>
-    <definedName name="Swap_Policy">'3 Build'!$B$16</definedName>
-    <definedName name="Swap_Pricer">'3 Build'!$B$19</definedName>
+    <definedName name="Swap_Policy">'3 Build'!$B$19</definedName>
+    <definedName name="Swap_Pricer">'3 Build'!$B$22</definedName>
     <definedName name="Swap_PV">'4 Results'!$B$7</definedName>
     <definedName name="Swap_Quote10">'2 Market'!$B$64</definedName>
     <definedName name="Swap_Quote11">'2 Market'!$B$67</definedName>
@@ -73,19 +75,19 @@
     <definedName name="Swap_Quote9">'2 Market'!$B$61</definedName>
     <definedName name="Swap_Quotes">Swap_Quote21</definedName>
     <definedName name="Swap_RateFrequency">'1 Inputs'!$B$18</definedName>
-    <definedName name="Swap_Request0">'3 Build'!$B$25</definedName>
-    <definedName name="Swap_Request1">'3 Build'!$B$31</definedName>
+    <definedName name="Swap_Request0">'3 Build'!$B$28</definedName>
+    <definedName name="Swap_Request1">'3 Build'!$B$34</definedName>
     <definedName name="Swap_Requests">'1 Inputs'!$A$24:$A$26</definedName>
-    <definedName name="Swap_Result">'3 Build'!$B$22</definedName>
+    <definedName name="Swap_Result">'3 Build'!$B$25</definedName>
     <definedName name="Swap_Side">'1 Inputs'!$B$15</definedName>
     <definedName name="Swap_SofrConfig">'2 Market'!$B$103</definedName>
-    <definedName name="Swap_SofrCurve">'3 Build'!$B$37</definedName>
+    <definedName name="Swap_SofrCurve">'3 Build'!$B$40</definedName>
     <definedName name="Swap_SofrDiscount">'4 Results'!$B$13</definedName>
     <definedName name="Swap_SofrForward">'4 Results'!$B$15</definedName>
     <definedName name="Swap_SofrQuotes">'2 Market'!$A$7:$A$14</definedName>
     <definedName name="Swap_Spread">'1 Inputs'!$B$10</definedName>
     <definedName name="Swap_Start">'1 Inputs'!$B$11</definedName>
-    <definedName name="Swap_Trade">'3 Build'!$B$13</definedName>
+    <definedName name="Swap_Trade">'3 Build'!$B$16</definedName>
     <definedName name="Swap_ValuationDate">'1 Inputs'!$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -185,7 +187,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Use a currency consistent with the selected market index.</t>
+          <t>This study prices a USD contract in the USD/SOFR context.</t>
         </r>
       </text>
     </comment>
@@ -198,7 +200,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>SOFR and ESTR are constructed on the Market tab.</t>
+          <t>SOFR projects this swap; ESTR has a separate comparison context.</t>
         </r>
       </text>
     </comment>
@@ -585,7 +587,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Use Actual360 / LogLinear / extrapolation for both curves.</t>
+          <t>USD/SOFR and EUR/ESTR use separate bootstrap collateral assumptions.</t>
         </r>
       </text>
     </comment>
@@ -611,7 +613,20 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Adds EUR without replacing the USD configuration.</t>
+          <t>An independent configuration collection for the EUR/ESTR context.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B109" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>EUR OIS quotes bootstrap under EUR/ESTR collateral in their own context.</t>
         </r>
       </text>
     </comment>
@@ -634,7 +649,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Builds the curves configured on Market.</t>
+          <t>Bootstraps SOFR under USD collateral; this context prices the swap.</t>
         </r>
       </text>
     </comment>
@@ -647,11 +662,24 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t>Bootstraps ESTR under EUR collateral for comparison only.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t>The contract contains dates, rates and indices.</t>
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0">
+    <comment ref="B16" authorId="0">
       <text>
         <r>
           <rPr>
@@ -664,7 +692,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B16" authorId="0">
+    <comment ref="B19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -677,7 +705,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B19" authorId="0">
+    <comment ref="B22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -690,7 +718,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B22" authorId="0">
+    <comment ref="B25" authorId="0">
       <text>
         <r>
           <rPr>
@@ -703,7 +731,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B25" authorId="0">
+    <comment ref="B28" authorId="0">
       <text>
         <r>
           <rPr>
@@ -716,7 +744,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B28" authorId="0">
+    <comment ref="B31" authorId="0">
       <text>
         <r>
           <rPr>
@@ -729,7 +757,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B31" authorId="0">
+    <comment ref="B34" authorId="0">
       <text>
         <r>
           <rPr>
@@ -742,7 +770,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B34" authorId="0">
+    <comment ref="B37" authorId="0">
       <text>
         <r>
           <rPr>
@@ -755,19 +783,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="B37" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Reusable curve object for point queries and node reports.</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="B40" authorId="0">
       <text>
         <r>
@@ -777,7 +792,20 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Reusable curve object for point queries and node reports.</t>
+          <t>Reads the curve from its matching collateral context.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B43" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Reads the curve from its matching collateral context.</t>
         </r>
       </text>
     </comment>
@@ -909,12 +937,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="210">
   <si>
     <t>Swap pricing · a guided example</t>
   </si>
   <si>
-    <t>Build USD SOFR and EUR ESTR curves, then value one receive-fixed USD swap.</t>
+    <t>Value one receive-fixed USD swap under USD/SOFR collateral. Build a separate EUR/ESTR market for curve comparisons.</t>
   </si>
   <si>
     <t>Before you start: load quantsupport.xll in 64-bit Windows Excel, then press Ctrl+Alt+F9. Results are blank until Excel calculates. Dates are ISO text; enter 4% as 0.04.</t>
@@ -1091,7 +1119,7 @@
     <t>USD</t>
   </si>
   <si>
-    <t>Use a currency consistent with the selected market index.</t>
+    <t>This study prices a USD contract in the USD/SOFR context.</t>
   </si>
   <si>
     <t>Projection index</t>
@@ -1100,7 +1128,7 @@
     <t>SOFR</t>
   </si>
   <si>
-    <t>SOFR and ESTR are constructed on the Market tab.</t>
+    <t>SOFR projects this swap; ESTR has a separate comparison context.</t>
   </si>
   <si>
     <t>Position side</t>
@@ -1334,10 +1362,10 @@
     <t>2.21 Load quote</t>
   </si>
   <si>
-    <t>3. Create curve configurations</t>
-  </si>
-  <si>
-    <t>Use Actual360 / LogLinear / extrapolation for both curves.</t>
+    <t>3. Create USD configurations</t>
+  </si>
+  <si>
+    <t>USD/SOFR and EUR/ESTR use separate bootstrap collateral assumptions.</t>
   </si>
   <si>
     <t>4. Configure SOFR</t>
@@ -1346,10 +1374,16 @@
     <t>Bootstraps the visible USD deposit / OIS quotes.</t>
   </si>
   <si>
-    <t>5. Configure ESTR</t>
-  </si>
-  <si>
-    <t>Adds EUR without replacing the USD configuration.</t>
+    <t>5. Create EUR configurations</t>
+  </si>
+  <si>
+    <t>An independent configuration collection for the EUR/ESTR context.</t>
+  </si>
+  <si>
+    <t>6. Configure ESTR</t>
+  </si>
+  <si>
+    <t>EUR OIS quotes bootstrap under EUR/ESTR collateral in their own context.</t>
   </si>
   <si>
     <t>Build the pricing objects</t>
@@ -1367,10 +1401,16 @@
     <t>Purpose</t>
   </si>
   <si>
-    <t>1. Initialize the context</t>
-  </si>
-  <si>
-    <t>Builds the curves configured on Market.</t>
+    <t>1.1 Initialize USD context</t>
+  </si>
+  <si>
+    <t>Bootstraps SOFR under USD collateral; this context prices the swap.</t>
+  </si>
+  <si>
+    <t>1.2 Initialize EUR context</t>
+  </si>
+  <si>
+    <t>Bootstraps ESTR under EUR collateral for comparison only.</t>
   </si>
   <si>
     <t>2. Define the instrument</t>
@@ -1427,7 +1467,7 @@
     <t>9. Inspect SOFR</t>
   </si>
   <si>
-    <t>Reusable curve object for point queries and node reports.</t>
+    <t>Reads the curve from its matching collateral context.</t>
   </si>
   <si>
     <t>9. Inspect ESTR</t>
@@ -2510,7 +2550,7 @@
       <c r="A13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C13" s="7" t="s">
@@ -2521,7 +2561,7 @@
       <c r="A14" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -2651,7 +2691,7 @@
     <tabColor rgb="FF337AB7"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="3" width="42.7109375" style="1" customWidth="1"/>
@@ -3324,7 +3364,7 @@
         <v>141</v>
       </c>
       <c r="B100" s="10" cm="1" t="str">
-        <f t="array" ref="B100">_xll.QS.CURVE.CONFIGS.CREATE("Swap.Curves")</f>
+        <f t="array" ref="B100">_xll.QS.CURVE.CONFIGS.CREATE("Swap.UsdCurves")</f>
         <v/>
       </c>
       <c r="C100" s="7" t="s">
@@ -3334,7 +3374,7 @@
     <row r="101" spans="1:3" ht="34" customHeight="1">
       <c r="A101" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B100),",",", ")</f>
-        <v>=QS.CURVE.CONFIGS.CREATE("Swap.Curves")</v>
+        <v>=QS.CURVE.CONFIGS.CREATE("Swap.UsdCurves")</v>
       </c>
       <c r="B101" s="13"/>
       <c r="C101" s="13"/>
@@ -3364,7 +3404,7 @@
         <v>145</v>
       </c>
       <c r="B106" s="10" cm="1" t="str">
-        <f t="array" ref="B106">_xll.QS.CURVE.CONFIGS.ADD(Swap_SofrConfig,"ESTR","Actual360","LogLinear",TRUE,Swap_EstrQuotes)</f>
+        <f t="array" ref="B106">_xll.QS.CURVE.CONFIGS.CREATE("Swap.EurCurves")</f>
         <v/>
       </c>
       <c r="C106" s="7" t="s">
@@ -3374,13 +3414,33 @@
     <row r="107" spans="1:3" ht="34" customHeight="1">
       <c r="A107" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B106),",",", ")</f>
-        <v>=QS.CURVE.CONFIGS.ADD(Swap_SofrConfig, "ESTR", "Actual360", "LogLinear", TRUE, Swap_EstrQuotes)</v>
+        <v>=QS.CURVE.CONFIGS.CREATE("Swap.EurCurves")</v>
       </c>
       <c r="B107" s="13"/>
       <c r="C107" s="13"/>
     </row>
+    <row r="109" spans="1:3" ht="38" customHeight="1">
+      <c r="A109" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B109" s="10" cm="1" t="str">
+        <f t="array" ref="B109">_xll.QS.CURVE.CONFIGS.ADD(Swap_InitialEstrCurves,"ESTR","Actual360","LogLinear",TRUE,Swap_EstrQuotes)</f>
+        <v/>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" ht="34" customHeight="1">
+      <c r="A110" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B109),",",", ")</f>
+        <v>=QS.CURVE.CONFIGS.ADD(Swap_InitialEstrCurves, "ESTR", "Actual360", "LogLinear", TRUE, Swap_EstrQuotes)</v>
+      </c>
+      <c r="B110" s="13"/>
+      <c r="C110" s="13"/>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C3"/>
     <mergeCell ref="A35:C35"/>
@@ -3408,6 +3468,7 @@
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="A104:C104"/>
     <mergeCell ref="A107:C107"/>
+    <mergeCell ref="A110:C110"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
@@ -3428,7 +3489,7 @@
     <tabColor rgb="FF78909C"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
@@ -3437,14 +3498,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3459,262 +3520,282 @@
         <v>39</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="36" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>116</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="38" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B7" s="10" cm="1" t="str">
-        <f t="array" ref="B7">_xll.QS.CONTEXT.CREATE("Swap.Context",Swap_Quotes,Swap_Curves,,,,,,,,,,Swap_Currency,Swap_Index,"Mid")</f>
+        <f t="array" ref="B7">_xll.QS.CONTEXT.CREATE("Swap.Context",Swap_Quotes,Swap_SofrConfig,,,,,,,,,,Swap_Currency,Swap_Index,"Mid")</f>
         <v/>
       </c>
       <c r="C7" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="34" customHeight="1">
       <c r="A8" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B7),",",", ")</f>
-        <v>=QS.CONTEXT.CREATE("Swap.Context", Swap_Quotes, Swap_Curves, , , , , , , , , , Swap_Currency, Swap_Index, "Mid")</v>
+        <v>=QS.CONTEXT.CREATE("Swap.Context", Swap_Quotes, Swap_SofrConfig, , , , , , , , , , Swap_Currency, Swap_Index, "Mid")</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
     </row>
     <row r="10" spans="1:3" ht="38" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B10" s="10" cm="1" t="str">
-        <f t="array" ref="B10">_xll.QS.INSTRUMENT.SWAP("Swap.Instrument",Swap_Start,Swap_Maturity,Swap_Currency,Swap_Index,Swap_Notional,Swap_FixedRate,Swap_Spread,Swap_DayCounter,Swap_Compounding,Swap_RateFrequency,Swap_FixedFrequency,Swap_FloatFrequency)</f>
+        <f t="array" ref="B10">_xll.QS.CONTEXT.CREATE("Swap.EstrContext",Swap_Quotes,Swap_EstrConfig,,,,,,,,,,"EUR","ESTR","Mid")</f>
         <v/>
       </c>
       <c r="C10" s="7" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="48" customHeight="1">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="34" customHeight="1">
       <c r="A11" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B10),",",", ")</f>
-        <v>=QS.INSTRUMENT.SWAP("Swap.Instrument", Swap_Start, Swap_Maturity, Swap_Currency, Swap_Index, Swap_Notional, Swap_FixedRate, Swap_Spread, Swap_DayCounter, Swap_Compounding, Swap_RateFrequency, Swap_FixedFrequency, Swap_FloatFrequency)</v>
+        <v>=QS.CONTEXT.CREATE("Swap.EstrContext", Swap_Quotes, Swap_EstrConfig, , , , , , , , , , "EUR", "ESTR", "Mid")</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
     </row>
     <row r="13" spans="1:3" ht="38" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B13" s="10" cm="1" t="str">
-        <f t="array" ref="B13">_xll.QS.TRADE.CREATE("Swap.Trade",Swap_Instrument,Swap_ValuationDate,Swap_Side)</f>
+        <f t="array" ref="B13">_xll.QS.INSTRUMENT.SWAP("Swap.Instrument",Swap_Start,Swap_Maturity,Swap_Currency,Swap_Index,Swap_Notional,Swap_FixedRate,Swap_Spread,Swap_DayCounter,Swap_Compounding,Swap_RateFrequency,Swap_FixedFrequency,Swap_FloatFrequency)</f>
         <v/>
       </c>
       <c r="C13" s="7" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="34" customHeight="1">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="48" customHeight="1">
       <c r="A14" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B13),",",", ")</f>
-        <v>=QS.TRADE.CREATE("Swap.Trade", Swap_Instrument, Swap_ValuationDate, Swap_Side)</v>
+        <v>=QS.INSTRUMENT.SWAP("Swap.Instrument", Swap_Start, Swap_Maturity, Swap_Currency, Swap_Index, Swap_Notional, Swap_FixedRate, Swap_Spread, Swap_DayCounter, Swap_Compounding, Swap_RateFrequency, Swap_FixedFrequency, Swap_FloatFrequency)</v>
       </c>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
     </row>
     <row r="16" spans="1:3" ht="38" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B16" s="10" cm="1" t="str">
-        <f t="array" ref="B16">_xll.QS.DISCOUNT.POLICY.CSA("Swap.Policy",Swap_Currency,Swap_Index)</f>
+        <f t="array" ref="B16">_xll.QS.TRADE.CREATE("Swap.Trade",Swap_Instrument,Swap_ValuationDate,Swap_Side)</f>
         <v/>
       </c>
       <c r="C16" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="34" customHeight="1">
       <c r="A17" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B16),",",", ")</f>
-        <v>=QS.DISCOUNT.POLICY.CSA("Swap.Policy", Swap_Currency, Swap_Index)</v>
+        <v>=QS.TRADE.CREATE("Swap.Trade", Swap_Instrument, Swap_ValuationDate, Swap_Side)</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
     </row>
     <row r="19" spans="1:3" ht="38" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B19" s="10" cm="1" t="str">
-        <f t="array" ref="B19">_xll.QS.PRICER.CREATE("Swap.Pricer","DiscountedCashflowPricer",Swap_Policy)</f>
+        <f t="array" ref="B19">_xll.QS.DISCOUNT.POLICY.CSA("Swap.Policy",Swap_Currency,Swap_Index)</f>
         <v/>
       </c>
       <c r="C19" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="34" customHeight="1">
       <c r="A20" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B19),",",", ")</f>
-        <v>=QS.PRICER.CREATE("Swap.Pricer", "DiscountedCashflowPricer", Swap_Policy)</v>
+        <v>=QS.DISCOUNT.POLICY.CSA("Swap.Policy", Swap_Currency, Swap_Index)</v>
       </c>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
     </row>
     <row r="22" spans="1:3" ht="38" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B22" s="10" cm="1" t="str">
-        <f t="array" ref="B22">_xll.QS.EVALUATE("Swap.Results",Swap_Pricer,Swap_Trade,Swap_Context,Swap_Requests)</f>
+        <f t="array" ref="B22">_xll.QS.PRICER.CREATE("Swap.Pricer","DiscountedCashflowPricer",Swap_Policy)</f>
         <v/>
       </c>
       <c r="C22" s="7" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="34" customHeight="1">
       <c r="A23" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B22),",",", ")</f>
-        <v>=QS.EVALUATE("Swap.Results", Swap_Pricer, Swap_Trade, Swap_Context, Swap_Requests)</v>
+        <v>=QS.PRICER.CREATE("Swap.Pricer", "DiscountedCashflowPricer", Swap_Policy)</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
     </row>
     <row r="25" spans="1:3" ht="38" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B25" s="10" cm="1" t="str">
-        <f t="array" ref="B25">_xll.QS.REQUEST.FAIR.RATE(0)</f>
+        <f t="array" ref="B25">_xll.QS.EVALUATE("Swap.Results",Swap_Pricer,Swap_Trade,Swap_Context,Swap_Requests)</f>
         <v/>
       </c>
       <c r="C25" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="34" customHeight="1">
       <c r="A26" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B25),",",", ")</f>
-        <v>=QS.REQUEST.FAIR.RATE(0)</v>
+        <v>=QS.EVALUATE("Swap.Results", Swap_Pricer, Swap_Trade, Swap_Context, Swap_Requests)</v>
       </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
     </row>
     <row r="28" spans="1:3" ht="38" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B28" s="10" cm="1" t="str">
-        <f t="array" ref="B28">_xll.QS.EVALUATE("Swap.Fair0",Swap_Pricer,Swap_Trade,Swap_Context,Swap_Request0)</f>
+        <f t="array" ref="B28">_xll.QS.REQUEST.FAIR.RATE(0)</f>
         <v/>
       </c>
       <c r="C28" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="34" customHeight="1">
       <c r="A29" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B28),",",", ")</f>
-        <v>=QS.EVALUATE("Swap.Fair0", Swap_Pricer, Swap_Trade, Swap_Context, Swap_Request0)</v>
+        <v>=QS.REQUEST.FAIR.RATE(0)</v>
       </c>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
     </row>
     <row r="31" spans="1:3" ht="38" customHeight="1">
       <c r="A31" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B31" s="10" cm="1" t="str">
-        <f t="array" ref="B31">_xll.QS.REQUEST.FAIR.RATE(1)</f>
+        <f t="array" ref="B31">_xll.QS.EVALUATE("Swap.Fair0",Swap_Pricer,Swap_Trade,Swap_Context,Swap_Request0)</f>
         <v/>
       </c>
       <c r="C31" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="34" customHeight="1">
       <c r="A32" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B31),",",", ")</f>
-        <v>=QS.REQUEST.FAIR.RATE(1)</v>
+        <v>=QS.EVALUATE("Swap.Fair0", Swap_Pricer, Swap_Trade, Swap_Context, Swap_Request0)</v>
       </c>
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
     </row>
     <row r="34" spans="1:3" ht="38" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B34" s="10" cm="1" t="str">
-        <f t="array" ref="B34">_xll.QS.EVALUATE("Swap.Fair1",Swap_Pricer,Swap_Trade,Swap_Context,Swap_Request1)</f>
+        <f t="array" ref="B34">_xll.QS.REQUEST.FAIR.RATE(1)</f>
         <v/>
       </c>
       <c r="C34" s="7" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="34" customHeight="1">
       <c r="A35" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B34),",",", ")</f>
-        <v>=QS.EVALUATE("Swap.Fair1", Swap_Pricer, Swap_Trade, Swap_Context, Swap_Request1)</v>
+        <v>=QS.REQUEST.FAIR.RATE(1)</v>
       </c>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
     </row>
     <row r="37" spans="1:3" ht="38" customHeight="1">
       <c r="A37" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B37" s="10" cm="1" t="str">
+        <f t="array" ref="B37">_xll.QS.EVALUATE("Swap.Fair1",Swap_Pricer,Swap_Trade,Swap_Context,Swap_Request1)</f>
+        <v/>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>171</v>
-      </c>
-      <c r="B37" s="10" cm="1" t="str">
-        <f t="array" ref="B37">_xll.QS.CURVE.GET(Swap_Context,"SOFR")</f>
-        <v/>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="34" customHeight="1">
       <c r="A38" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B37),",",", ")</f>
-        <v>=QS.CURVE.GET(Swap_Context, "SOFR")</v>
+        <v>=QS.EVALUATE("Swap.Fair1", Swap_Pricer, Swap_Trade, Swap_Context, Swap_Request1)</v>
       </c>
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
     </row>
     <row r="40" spans="1:3" ht="38" customHeight="1">
       <c r="A40" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B40" s="10" cm="1" t="str">
-        <f t="array" ref="B40">_xll.QS.CURVE.GET(Swap_Context,"ESTR")</f>
+        <f t="array" ref="B40">_xll.QS.CURVE.GET(Swap_Context,"SOFR")</f>
         <v/>
       </c>
       <c r="C40" s="7" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="34" customHeight="1">
       <c r="A41" s="13" t="str">
         <f>SUBSTITUTE(_xlfn.FORMULATEXT(B40),",",", ")</f>
-        <v>=QS.CURVE.GET(Swap_Context, "ESTR")</v>
+        <v>=QS.CURVE.GET(Swap_Context, "SOFR")</v>
       </c>
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
     </row>
+    <row r="43" spans="1:3" ht="38" customHeight="1">
+      <c r="A43" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B43" s="10" cm="1" t="str">
+        <f t="array" ref="B43">_xll.QS.CURVE.GET(Swap_EstrContext,"ESTR")</f>
+        <v/>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="34" customHeight="1">
+      <c r="A44" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B43),",",", ")</f>
+        <v>=QS.CURVE.GET(Swap_EstrContext, "ESTR")</v>
+      </c>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C3"/>
     <mergeCell ref="A8:C8"/>
@@ -3729,6 +3810,7 @@
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A44:C44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
@@ -3759,14 +3841,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3781,118 +3863,118 @@
         <v>39</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="36" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="34" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B7" s="14" cm="1" t="str">
         <f t="array" ref="B7">_xll.QS.RESULT.VALUE(Swap_Result)</f>
         <v/>
       </c>
       <c r="C7" s="7" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="34" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B8" s="15" cm="1" t="str">
         <f t="array" ref="B8">_xll.QS.RESULT.FAIR.RATE(Swap_Fair0)</f>
         <v/>
       </c>
       <c r="C8" s="7" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="34" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B9" s="15" cm="1" t="str">
         <f t="array" ref="B9">_xll.QS.RESULT.FAIR.RATE(Swap_Fair1)</f>
         <v/>
       </c>
       <c r="C9" s="7" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="36" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="34" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B13" s="16" cm="1" t="str">
         <f t="array" ref="B13">_xll.QS.CURVE.DISCOUNT(Swap_SofrCurve,Swap_Maturity)</f>
         <v/>
       </c>
       <c r="C13" s="7" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="34" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B14" s="16" cm="1" t="str">
         <f t="array" ref="B14">_xll.QS.CURVE.DISCOUNT(Swap_EstrCurve,Swap_Maturity)</f>
         <v/>
       </c>
       <c r="C14" s="7" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="34" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B15" s="15" cm="1" t="str">
         <f t="array" ref="B15">_xll.QS.CURVE.FORWARD(Swap_SofrCurve,Swap_Start,Swap_Maturity,"Simple","Annual")</f>
         <v/>
       </c>
       <c r="C15" s="7" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="34" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B16" s="15" cm="1" t="str">
         <f t="array" ref="B16">_xll.QS.CURVE.FORWARD(Swap_EstrCurve,Swap_Start,Swap_Maturity,"Simple","Annual")</f>
         <v/>
       </c>
       <c r="C16" s="7" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="24" customHeight="1">
       <c r="A20" s="6" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3935,7 +4017,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3948,7 +4030,7 @@
     </row>
     <row r="2" spans="1:9" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3975,7 +4057,7 @@
         <v>39</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="24" customHeight="1">
@@ -4017,14 +4099,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4039,7 +4121,7 @@
         <v>39</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="24" customHeight="1">
@@ -4082,7 +4164,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="38" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4091,7 +4173,7 @@
     </row>
     <row r="2" spans="1:5" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4112,7 +4194,7 @@
     </row>
     <row r="6" spans="1:5" ht="24" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -4127,7 +4209,7 @@
     </row>
     <row r="26" spans="1:5" ht="24" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>

</xml_diff>